<commit_message>
espectros del 2018 y 219, todos funcionan c:
</commit_message>
<xml_diff>
--- a/Datos ESPARTACO/Parámetros para análisis de Antares/Resultados absorción cobalto 2018 y 2019.xlsx
+++ b/Datos ESPARTACO/Parámetros para análisis de Antares/Resultados absorción cobalto 2018 y 2019.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,20 +456,25 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Velocidad [km/s]</t>
+          <t>Velocidad obs. [km/s]</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Velocidad heliocéntrica [km/s]</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Profundidad / Altura</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>FWHM [Å]</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>EW [Å]</t>
         </is>
@@ -501,13 +506,16 @@
         <v>19.71</v>
       </c>
       <c r="G2" t="n">
+        <v>-3.12</v>
+      </c>
+      <c r="H2" t="n">
         <v>0.5629</v>
       </c>
-      <c r="H2" t="n">
-        <v>0.9429999999999999</v>
-      </c>
       <c r="I2" t="n">
-        <v>0.6163</v>
+        <v>0.9419999999999999</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.6153999999999999</v>
       </c>
     </row>
     <row r="3">
@@ -536,13 +544,16 @@
         <v>19.4</v>
       </c>
       <c r="G3" t="n">
-        <v>0.5504</v>
+        <v>-4.47</v>
       </c>
       <c r="H3" t="n">
-        <v>0.959</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="I3" t="n">
-        <v>0.6089</v>
+        <v>0.963</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.6576</v>
       </c>
     </row>
     <row r="4">
@@ -571,13 +582,16 @@
         <v>23.47</v>
       </c>
       <c r="G4" t="n">
+        <v>-2.53</v>
+      </c>
+      <c r="H4" t="n">
         <v>0.5656</v>
       </c>
-      <c r="H4" t="n">
-        <v>0.929</v>
-      </c>
       <c r="I4" t="n">
-        <v>0.6011</v>
+        <v>0.928</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.6006</v>
       </c>
     </row>
     <row r="5">
@@ -606,13 +620,16 @@
         <v>24.06</v>
       </c>
       <c r="G5" t="n">
-        <v>0.5551</v>
+        <v>-2.53</v>
       </c>
       <c r="H5" t="n">
-        <v>0.89</v>
+        <v>0.5595</v>
       </c>
       <c r="I5" t="n">
-        <v>0.5620000000000001</v>
+        <v>0.846</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.536</v>
       </c>
     </row>
     <row r="6">
@@ -641,13 +658,16 @@
         <v>24.2</v>
       </c>
       <c r="G6" t="n">
-        <v>0.5483</v>
+        <v>-3.38</v>
       </c>
       <c r="H6" t="n">
-        <v>0.913</v>
+        <v>0.5556</v>
       </c>
       <c r="I6" t="n">
-        <v>0.6128</v>
+        <v>0.873</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.5994</v>
       </c>
     </row>
     <row r="7">
@@ -676,13 +696,16 @@
         <v>25.74</v>
       </c>
       <c r="G7" t="n">
-        <v>0.5524</v>
+        <v>-2.45</v>
       </c>
       <c r="H7" t="n">
-        <v>0.848</v>
+        <v>0.5563</v>
       </c>
       <c r="I7" t="n">
-        <v>0.5523</v>
+        <v>0.824</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.5276</v>
       </c>
     </row>
     <row r="8">
@@ -711,12 +734,15 @@
         <v>26.07</v>
       </c>
       <c r="G8" t="n">
+        <v>-3.14</v>
+      </c>
+      <c r="H8" t="n">
         <v>0.5606</v>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
         <v>0.896</v>
       </c>
-      <c r="I8" t="n">
+      <c r="J8" t="n">
         <v>0.6126</v>
       </c>
     </row>
@@ -746,13 +772,16 @@
         <v>26.94</v>
       </c>
       <c r="G9" t="n">
-        <v>0.5601</v>
+        <v>-2.53</v>
       </c>
       <c r="H9" t="n">
-        <v>0.875</v>
+        <v>0.5613</v>
       </c>
       <c r="I9" t="n">
-        <v>0.6022999999999999</v>
+        <v>0.862</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.5947</v>
       </c>
     </row>
     <row r="10">
@@ -781,13 +810,16 @@
         <v>26.66</v>
       </c>
       <c r="G10" t="n">
-        <v>0.5605</v>
+        <v>-2.7</v>
       </c>
       <c r="H10" t="n">
-        <v>0.967</v>
+        <v>0.5615</v>
       </c>
       <c r="I10" t="n">
-        <v>0.6563</v>
+        <v>0.961</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.6451</v>
       </c>
     </row>
     <row r="11">
@@ -816,13 +848,16 @@
         <v>22.5</v>
       </c>
       <c r="G11" t="n">
-        <v>0.5322</v>
+        <v>-3.74</v>
       </c>
       <c r="H11" t="n">
-        <v>0.961</v>
+        <v>0.5371</v>
       </c>
       <c r="I11" t="n">
-        <v>0.6093</v>
+        <v>0.9419999999999999</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.5981</v>
       </c>
     </row>
   </sheetData>

</xml_diff>